<commit_message>
added email implementation readiness
</commit_message>
<xml_diff>
--- a/docs/hebrew-review.xlsx
+++ b/docs/hebrew-review.xlsx
@@ -7889,16 +7889,26 @@
     <t>email.verifyEmail.text</t>
   </si>
   <si>
-    <t>Hello Dana,
+    <t>Verify your email
+Hi Dana,
 To finish signing up, please verify your email address.
-Verify email: https://events.example.com/…
-This link works for 24 hours. If you didn't sign up for Event Planner, you can ignore this email.</t>
-  </si>
-  <si>
-    <t>שלום Dana,
+Verify Email: https://events.example.com/…
+This link works for 24 hours.
+Thanks,
+Event Planner
+This email was sent securely by Event Planner.
+If you didn't sign up for Event Planner, you can safely ignore this email.</t>
+  </si>
+  <si>
+    <t>אימות כתובת האימייל
+שלום ⁨Dana⁩,
 כדי להשלים את ההרשמה, יש לאמת את כתובת האימייל שלך.
 אימות האימייל: https://events.example.com/…
-הקישור תקף ל-24 שעות. אם לא נרשמת ל-Event Planner, אפשר להתעלם מהודעה זו.</t>
+הקישור תקף ל-24 שעות.
+תודה,
+Event Planner
+ההודעה נשלחה באופן מאובטח על ידי Event Planner.
+אם לא נרשמת ל-Event Planner, אפשר להתעלם מהודעה זו בבטחה.</t>
   </si>
   <si>
     <t>email.resetPassword.subject</t>
@@ -7913,16 +7923,26 @@
     <t>email.resetPassword.text</t>
   </si>
   <si>
-    <t>Hello Dana,
+    <t>Reset your password
+Hi Dana,
 We received a request to reset the password of your account.
-Choose a new password: https://events.example.com/…
-This link works for 60 minutes, once. If you didn't ask to reset your password, you can ignore this email; your password stays the same.</t>
-  </si>
-  <si>
-    <t>שלום Dana,
+Choose a New Password: https://events.example.com/…
+This link works for 60 minutes, once.
+Thanks,
+Event Planner
+This email was sent securely by Event Planner.
+If you didn't ask to reset your password, you can safely ignore this email; your password stays the same.</t>
+  </si>
+  <si>
+    <t>איפוס הסיסמה
+שלום ⁨Dana⁩,
 התקבלה בקשה לאפס את הסיסמה של החשבון שלך.
 בחירת סיסמה חדשה: https://events.example.com/…
-הקישור תקף ל-60 דקות ולשימוש אחד. אם לא ביקשת לאפס את הסיסמה, אפשר להתעלם מהודעה זו; הסיסמה לא תשתנה.</t>
+הקישור תקף ל-60 דקות ולשימוש אחד.
+תודה,
+Event Planner
+ההודעה נשלחה באופן מאובטח על ידי Event Planner.
+אם לא ביקשת לאפס את הסיסמה, אפשר להתעלם מהודעה זו בבטחה; הסיסמה לא תשתנה.</t>
   </si>
   <si>
     <t>email.invitation.subject</t>
@@ -7931,22 +7951,38 @@
     <t>You're invited to "Garden Party" on Event Planner</t>
   </si>
   <si>
-    <t>הוזמנת לאירוע "Garden Party" ב-Event Planner</t>
+    <t>הוזמנת לאירוע "⁨Garden Party⁩" ב-Event Planner</t>
   </si>
   <si>
     <t>email.invitation.text</t>
   </si>
   <si>
-    <t>Riley invited you to the event "Garden Party" as Admin.
-To get access, sign up to Event Planner with this email address.
-Sign up: https://events.example.com/…
-If you weren't expecting this invitation, you can ignore this email.</t>
-  </si>
-  <si>
-    <t>Riley הזמין/ה אותך לאירוע "Garden Party" בהרשאת מנהל.
-כדי לקבל גישה, יש להירשם ל-Event Planner עם כתובת האימייל הזו.
-הרשמה: https://events.example.com/…
-אם לא ציפית להזמנה הזו, אפשר להתעלם מהודעה זו.</t>
+    <t>You're invited to Garden Party
+Hi,
+Riley invited you to collaborate on Garden Party.
+Role: Admin
+Date: October 24, 2026
+Accept Invitation: https://events.example.com/…
+Once accepted, the event will appear in your My Events page.
+If you don't have an account yet, you can create one using this email address.
+Thanks,
+Event Planner
+This invitation was sent securely by Event Planner.
+If you weren't expecting this, you can safely ignore this email.</t>
+  </si>
+  <si>
+    <t>הוזמנת לאירוע ⁨Garden Party⁩
+שלום,
+⁨Riley⁩ הזמין/ה אותך להצטרף לניהול האירוע ⁨Garden Party⁩.
+הרשאה: מנהל
+תאריך: 24 באוקטובר 2026
+קבלת ההזמנה: https://events.example.com/…
+לאחר קבלת ההזמנה, האירוע יופיע בדף "האירועים שלי".
+אם עדיין אין לך חשבון, אפשר ליצור אותו עם כתובת האימייל הזו.
+תודה,
+Event Planner
+ההזמנה נשלחה באופן מאובטח על ידי Event Planner.
+אם לא ציפית להודעה הזו, אפשר להתעלם ממנה בבטחה.</t>
   </si>
   <si>
     <t>email.accessGranted.subject</t>
@@ -7955,20 +7991,36 @@
     <t>You now have access to "Garden Party"</t>
   </si>
   <si>
-    <t>קיבלת גישה לאירוע "Garden Party"</t>
+    <t>קיבלת גישה לאירוע "⁨Garden Party⁩"</t>
   </si>
   <si>
     <t>email.accessGranted.text</t>
   </si>
   <si>
-    <t>Riley gave you access to the event "Garden Party" as Admin.
-Open the event: https://events.example.com/…
-The event now appears in your list of events.</t>
-  </si>
-  <si>
-    <t>Riley נתן/ה לך גישה לאירוע "Garden Party" בהרשאת מנהל.
+    <t>You now have access to Garden Party
+Hi Dana,
+Riley gave you access to Garden Party.
+Role: Admin
+Date: October 24, 2026
+Open Event: https://events.example.com/…
+The event now appears in your My Events page.
+Thanks,
+Event Planner
+This email was sent securely by Event Planner.
+If you weren't expecting this, you can safely ignore this email.</t>
+  </si>
+  <si>
+    <t>קיבלת גישה לאירוע ⁨Garden Party⁩
+שלום ⁨Dana⁩,
+⁨Riley⁩ נתן/ה לך גישה לאירוע ⁨Garden Party⁩.
+הרשאה: מנהל
+תאריך: 24 באוקטובר 2026
 פתיחת האירוע: https://events.example.com/…
-האירוע מופיע עכשיו ברשימת האירועים שלך.</t>
+האירוע מופיע עכשיו בדף "האירועים שלי".
+תודה,
+Event Planner
+ההודעה נשלחה באופן מאובטח על ידי Event Planner.
+אם לא ציפית להודעה הזו, אפשר להתעלם ממנה בבטחה.</t>
   </si>
   <si>
     <t>email.testEmail.subject</t>
@@ -7983,13 +8035,21 @@
     <t>email.testEmail.text</t>
   </si>
   <si>
-    <t>This is a test email. If it arrived, sending email works.
+    <t>Sending email works
+This is a test email. If it arrived, sending email works.
 Open Event Planner: https://events.example.com/…
+Thanks,
+Event Planner
+This email was sent securely by Event Planner.
 Sent from the System page by a Super User.</t>
   </si>
   <si>
-    <t>זהו אימייל בדיקה. אם הוא הגיע, שליחת האימיילים עובדת.
+    <t>שליחת אימיילים עובדת
+זהו אימייל בדיקה. אם הוא הגיע, שליחת האימיילים עובדת.
 פתיחת Event Planner: https://events.example.com/…
+תודה,
+Event Planner
+ההודעה נשלחה באופן מאובטח על ידי Event Planner.
 נשלח מדף המערכת על ידי משתמש-על.</t>
   </si>
   <si>

</xml_diff>

<commit_message>
fixed some issues with Evnet Layout Table Arrangements and to Tables tab
</commit_message>
<xml_diff>
--- a/docs/hebrew-review.xlsx
+++ b/docs/hebrew-review.xlsx
@@ -6734,10 +6734,10 @@
     <t>layout.warnings.none</t>
   </si>
   <si>
-    <t>No capacity warnings.</t>
-  </si>
-  <si>
-    <t>אין אזהרות קיבולת.</t>
+    <t>No tables over capacity.</t>
+  </si>
+  <si>
+    <t>אין שולחנות בחריגה מהקיבולת.</t>
   </si>
   <si>
     <t>layout.selected.title</t>
@@ -7211,10 +7211,10 @@
     <t>בר</t>
   </si>
   <si>
-    <t>layout.objects.STEPS</t>
-  </si>
-  <si>
-    <t>Steps</t>
+    <t>layout.objects.STAIRS</t>
+  </si>
+  <si>
+    <t>Stairs</t>
   </si>
   <si>
     <t>מדרגות</t>
@@ -7583,10 +7583,10 @@
     <t>layout.arrangement.inspector.labelHint</t>
   </si>
   <si>
-    <t>Shown instead of the kind, such as Dance floor.</t>
-  </si>
-  <si>
-    <t>מוצגת במקום סוג הפריט, למשל רחבת ריקודים.</t>
+    <t>Shown instead of the kind, such as Dance floor or Stairs to the balcony.</t>
+  </si>
+  <si>
+    <t>מוצגת במקום סוג הפריט, למשל רחבת ריקודים או מדרגות ליציע.</t>
   </si>
   <si>
     <t>layout.arrangement.inspector.unplace</t>

</xml_diff>